<commit_message>
ALPS: replace QR with CPU eigh (match original algorithm)
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/剪枝结果-飞书.xlsx
+++ b/剪枝结果-飞书.xlsx
@@ -5053,7 +5053,9 @@
       <c r="G6" s="20" t="n"/>
       <c r="H6" s="20" t="n"/>
       <c r="I6" s="20" t="n"/>
-      <c r="J6" s="20" t="n"/>
+      <c r="J6" s="20" t="n">
+        <v>8.381324807831589</v>
+      </c>
       <c r="K6" s="18" t="inlineStr">
         <is>
           <t>N/A</t>

</xml_diff>

<commit_message>
update res and sth about device map
</commit_message>
<xml_diff>
--- a/剪枝结果-飞书.xlsx
+++ b/剪枝结果-飞书.xlsx
@@ -2643,15 +2643,33 @@
           <t>2:4</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="14" t="n"/>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="14" t="n"/>
-      <c r="H8" s="14" t="n"/>
-      <c r="I8" s="14" t="n"/>
-      <c r="J8" s="14" t="n"/>
+      <c r="B8" s="14" t="n">
+        <v>0.8381999999999999</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>0.8087</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>0.6251</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>0.6526999999999999</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>0.6965</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>0.4369</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>0.6369</v>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>14.98162884162644</v>
+      </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -2684,15 +2702,33 @@
           <t>4:8</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="14" t="n"/>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
-      <c r="I9" s="14" t="n"/>
-      <c r="J9" s="14" t="n"/>
+      <c r="B9" s="14" t="n">
+        <v>0.8517</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>0.7762</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>0.6879</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>0.6827</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>0.7546</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>0.4838</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>0.422</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>0.6656</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>10.17508977614515</v>
+      </c>
       <c r="K9" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -2929,8 +2965,12 @@
       <c r="M14" s="15" t="n">
         <v>79.08</v>
       </c>
-      <c r="N14" s="8" t="n"/>
-      <c r="O14" s="8" t="n"/>
+      <c r="N14" s="15" t="n">
+        <v>77.68287677743521</v>
+      </c>
+      <c r="O14" s="15" t="n">
+        <v>80.81821919435879</v>
+      </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
@@ -3023,8 +3063,12 @@
       <c r="M16" s="15" t="n">
         <v>56.96</v>
       </c>
-      <c r="N16" s="8" t="n"/>
-      <c r="O16" s="8" t="n"/>
+      <c r="N16" s="15" t="n">
+        <v>71.32275884415212</v>
+      </c>
+      <c r="O16" s="15" t="n">
+        <v>71.93268971103802</v>
+      </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -3068,8 +3112,12 @@
       <c r="M17" s="15" t="n">
         <v>64.28</v>
       </c>
-      <c r="N17" s="8" t="n"/>
-      <c r="O17" s="8" t="n"/>
+      <c r="N17" s="15" t="n">
+        <v>76.07087491557432</v>
+      </c>
+      <c r="O17" s="15" t="n">
+        <v>75.57371872889358</v>
+      </c>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -3393,15 +3441,33 @@
           <t>2:4</t>
         </is>
       </c>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="14" t="n"/>
-      <c r="F24" s="14" t="n"/>
-      <c r="G24" s="14" t="n"/>
-      <c r="H24" s="14" t="n"/>
-      <c r="I24" s="14" t="n"/>
-      <c r="J24" s="14" t="n"/>
+      <c r="B24" s="14" t="n">
+        <v>0.8217</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>0.6029</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>0.5586</v>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>0.6306</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>0.6961000000000001</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>0.4181</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>0.338</v>
+      </c>
+      <c r="I24" s="14" t="n">
+        <v>0.5809</v>
+      </c>
+      <c r="J24" s="14" t="n">
+        <v>15.40946848894207</v>
+      </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -3434,15 +3500,33 @@
           <t>4:8</t>
         </is>
       </c>
-      <c r="B25" s="14" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="14" t="n"/>
-      <c r="I25" s="14" t="n"/>
-      <c r="J25" s="14" t="n"/>
+      <c r="B25" s="14" t="n">
+        <v>0.848</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>0.7256</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>0.6191</v>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>0.6606</v>
+      </c>
+      <c r="F25" s="14" t="n">
+        <v>0.7609</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>0.4812</v>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>0.372</v>
+      </c>
+      <c r="I25" s="14" t="n">
+        <v>0.6382</v>
+      </c>
+      <c r="J25" s="14" t="n">
+        <v>12.49607959892532</v>
+      </c>
       <c r="K25" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -3523,11 +3607,21 @@
       <c r="J27" s="14" t="n">
         <v>7.855145447281187</v>
       </c>
-      <c r="K27" s="7" t="n"/>
-      <c r="L27" s="7" t="n"/>
-      <c r="M27" s="7" t="n"/>
-      <c r="N27" s="7" t="n"/>
-      <c r="O27" s="7" t="n"/>
+      <c r="K27" s="14" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="L27" s="14" t="n">
+        <v>82.968</v>
+      </c>
+      <c r="M27" s="14" t="n">
+        <v>83.36</v>
+      </c>
+      <c r="N27" s="14" t="n">
+        <v>83.11612778481857</v>
+      </c>
+      <c r="O27" s="14" t="n">
+        <v>84.03603194620464</v>
+      </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
@@ -6745,15 +6839,33 @@
           <t>2:4</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="14" t="n"/>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="14" t="n"/>
-      <c r="H8" s="14" t="n"/>
-      <c r="I8" s="14" t="n"/>
-      <c r="J8" s="14" t="n"/>
+      <c r="B8" s="14" t="n">
+        <v>0.8547</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>0.8051</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>0.6685</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>0.6796</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>0.7066</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>0.4497</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>0.6535</v>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>11.0829279186429</v>
+      </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -6786,15 +6898,33 @@
           <t>4:8</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="14" t="n"/>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
-      <c r="I9" s="14" t="n"/>
-      <c r="J9" s="14" t="n"/>
+      <c r="B9" s="14" t="n">
+        <v>0.8522999999999999</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>0.8014</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>0.7105</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>0.6796</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>0.7534</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>0.5077</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>0.6778</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>9.589240670634753</v>
+      </c>
       <c r="K9" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -7031,8 +7161,12 @@
       <c r="M14" s="15" t="n">
         <v>66.12</v>
       </c>
-      <c r="N14" s="8" t="n"/>
-      <c r="O14" s="8" t="n"/>
+      <c r="N14" s="15" t="n">
+        <v>75.76339063864515</v>
+      </c>
+      <c r="O14" s="15" t="n">
+        <v>76.27134765966129</v>
+      </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
@@ -7125,8 +7259,12 @@
       <c r="M16" s="15" t="n">
         <v>48.6</v>
       </c>
-      <c r="N16" s="8" t="n"/>
-      <c r="O16" s="8" t="n"/>
+      <c r="N16" s="15" t="n">
+        <v>70.94698961418374</v>
+      </c>
+      <c r="O16" s="15" t="n">
+        <v>69.11274740354594</v>
+      </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -7170,8 +7308,12 @@
       <c r="M17" s="15" t="n">
         <v>45.12</v>
       </c>
-      <c r="N17" s="8" t="n"/>
-      <c r="O17" s="8" t="n"/>
+      <c r="N17" s="15" t="n">
+        <v>74.18798261259997</v>
+      </c>
+      <c r="O17" s="15" t="n">
+        <v>69.34299565314998</v>
+      </c>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -7495,15 +7637,33 @@
           <t>2:4</t>
         </is>
       </c>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="14" t="n"/>
-      <c r="F24" s="14" t="n"/>
-      <c r="G24" s="14" t="n"/>
-      <c r="H24" s="14" t="n"/>
-      <c r="I24" s="14" t="n"/>
-      <c r="J24" s="14" t="n"/>
+      <c r="B24" s="14" t="n">
+        <v>0.8012</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>0.6462</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>0.6036</v>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>0.6551</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>0.7113</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>0.4437</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>0.374</v>
+      </c>
+      <c r="I24" s="14" t="n">
+        <v>0.605</v>
+      </c>
+      <c r="J24" s="14" t="n">
+        <v>13.86627246312579</v>
+      </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -7536,15 +7696,33 @@
           <t>4:8</t>
         </is>
       </c>
-      <c r="B25" s="14" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="14" t="n"/>
-      <c r="I25" s="14" t="n"/>
-      <c r="J25" s="14" t="n"/>
+      <c r="B25" s="14" t="n">
+        <v>0.8453000000000001</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>0.6715</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>0.6445</v>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>0.6803</v>
+      </c>
+      <c r="F25" s="14" t="n">
+        <v>0.7521</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>0.4974</v>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>0.384</v>
+      </c>
+      <c r="I25" s="14" t="n">
+        <v>0.6393</v>
+      </c>
+      <c r="J25" s="14" t="n">
+        <v>12.06350600064571</v>
+      </c>
       <c r="K25" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -7625,11 +7803,21 @@
       <c r="J27" s="14" t="n">
         <v>7.855145447281187</v>
       </c>
-      <c r="K27" s="7" t="n"/>
-      <c r="L27" s="7" t="n"/>
-      <c r="M27" s="7" t="n"/>
-      <c r="N27" s="7" t="n"/>
-      <c r="O27" s="7" t="n"/>
+      <c r="K27" s="14" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="L27" s="14" t="n">
+        <v>82.968</v>
+      </c>
+      <c r="M27" s="14" t="n">
+        <v>83.36</v>
+      </c>
+      <c r="N27" s="14" t="n">
+        <v>83.11612778481857</v>
+      </c>
+      <c r="O27" s="14" t="n">
+        <v>84.03603194620464</v>
+      </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
@@ -10797,15 +10985,33 @@
           <t>2:4</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="14" t="n"/>
-      <c r="D8" s="14" t="n"/>
-      <c r="E8" s="14" t="n"/>
-      <c r="F8" s="14" t="n"/>
-      <c r="G8" s="14" t="n"/>
-      <c r="H8" s="14" t="n"/>
-      <c r="I8" s="14" t="n"/>
-      <c r="J8" s="14" t="n"/>
+      <c r="B8" s="14" t="n">
+        <v>0.8544</v>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>0.8159</v>
+      </c>
+      <c r="D8" s="14" t="n">
+        <v>0.6835</v>
+      </c>
+      <c r="E8" s="14" t="n">
+        <v>0.6851</v>
+      </c>
+      <c r="F8" s="14" t="n">
+        <v>0.7302</v>
+      </c>
+      <c r="G8" s="14" t="n">
+        <v>0.4795</v>
+      </c>
+      <c r="H8" s="14" t="n">
+        <v>0.414</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>0.6661</v>
+      </c>
+      <c r="J8" s="14" t="n">
+        <v>10.47040152304533</v>
+      </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -10838,15 +11044,33 @@
           <t>4:8</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="14" t="n"/>
-      <c r="D9" s="14" t="n"/>
-      <c r="E9" s="14" t="n"/>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-      <c r="H9" s="14" t="n"/>
-      <c r="I9" s="14" t="n"/>
-      <c r="J9" s="14" t="n"/>
+      <c r="B9" s="14" t="n">
+        <v>0.8587</v>
+      </c>
+      <c r="C9" s="14" t="n">
+        <v>0.7653</v>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>0.718</v>
+      </c>
+      <c r="E9" s="14" t="n">
+        <v>0.7017</v>
+      </c>
+      <c r="F9" s="14" t="n">
+        <v>0.7778</v>
+      </c>
+      <c r="G9" s="14" t="n">
+        <v>0.5239</v>
+      </c>
+      <c r="H9" s="14" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>0.6836</v>
+      </c>
+      <c r="J9" s="14" t="n">
+        <v>9.209013861652336</v>
+      </c>
       <c r="K9" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -11080,9 +11304,15 @@
       <c r="L14" s="15" t="n">
         <v>80.404</v>
       </c>
-      <c r="M14" s="8" t="n"/>
-      <c r="N14" s="8" t="n"/>
-      <c r="O14" s="8" t="n"/>
+      <c r="M14" s="15" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="N14" s="15" t="n">
+        <v>76.20438550953283</v>
+      </c>
+      <c r="O14" s="15" t="n">
+        <v>75.33209637738319</v>
+      </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
@@ -11140,37 +11370,47 @@
         </is>
       </c>
       <c r="B16" s="14" t="n">
-        <v>0.8483000000000001</v>
+        <v>0.8425</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>0.8339</v>
+        <v>0.8375</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>0.6375</v>
+        <v>0.6344</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0.6701</v>
+        <v>0.6796</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>0.5939</v>
+        <v>0.5783</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>0.3686</v>
+        <v>0.3626</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.364</v>
+        <v>0.362</v>
       </c>
       <c r="I16" s="14" t="n">
-        <v>0.6166</v>
+        <v>0.6138</v>
       </c>
       <c r="J16" s="14" t="n">
-        <v>12.17765478688282</v>
-      </c>
-      <c r="K16" s="8" t="n"/>
-      <c r="L16" s="8" t="n"/>
-      <c r="M16" s="8" t="n"/>
-      <c r="N16" s="8" t="n"/>
-      <c r="O16" s="8" t="n"/>
+        <v>11.90872614135452</v>
+      </c>
+      <c r="K16" s="15" t="n">
+        <v>77.5</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>76.60600000000001</v>
+      </c>
+      <c r="M16" s="15" t="n">
+        <v>51.64</v>
+      </c>
+      <c r="N16" s="15" t="n">
+        <v>70.57294975750568</v>
+      </c>
+      <c r="O16" s="15" t="n">
+        <v>69.07973743937642</v>
+      </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
@@ -11178,20 +11418,48 @@
           <t>4:8</t>
         </is>
       </c>
-      <c r="B17" s="14" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
-      <c r="E17" s="14" t="n"/>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="14" t="n"/>
-      <c r="H17" s="14" t="n"/>
-      <c r="I17" s="14" t="n"/>
-      <c r="J17" s="14" t="n"/>
-      <c r="K17" s="8" t="n"/>
-      <c r="L17" s="8" t="n"/>
-      <c r="M17" s="8" t="n"/>
-      <c r="N17" s="8" t="n"/>
-      <c r="O17" s="8" t="n"/>
+      <c r="B17" s="14" t="n">
+        <v>0.8547</v>
+      </c>
+      <c r="C17" s="14" t="n">
+        <v>0.8339</v>
+      </c>
+      <c r="D17" s="14" t="n">
+        <v>0.6754</v>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>0.6756</v>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>0.6263</v>
+      </c>
+      <c r="G17" s="14" t="n">
+        <v>0.4078</v>
+      </c>
+      <c r="H17" s="14" t="n">
+        <v>0.392</v>
+      </c>
+      <c r="I17" s="14" t="n">
+        <v>0.638</v>
+      </c>
+      <c r="J17" s="14" t="n">
+        <v>10.8883927478228</v>
+      </c>
+      <c r="K17" s="15" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="L17" s="15" t="n">
+        <v>76.392</v>
+      </c>
+      <c r="M17" s="15" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="N17" s="15" t="n">
+        <v>74.94787703326428</v>
+      </c>
+      <c r="O17" s="15" t="n">
+        <v>69.58496925831606</v>
+      </c>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
@@ -11515,15 +11783,33 @@
           <t>2:4</t>
         </is>
       </c>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="14" t="n"/>
-      <c r="F24" s="14" t="n"/>
-      <c r="G24" s="14" t="n"/>
-      <c r="H24" s="14" t="n"/>
-      <c r="I24" s="14" t="n"/>
-      <c r="J24" s="14" t="n"/>
+      <c r="B24" s="14" t="n">
+        <v>0.8324</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>0.704</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>0.6237</v>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>0.6717</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>0.7214</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>0.4582</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>0.394</v>
+      </c>
+      <c r="I24" s="14" t="n">
+        <v>0.6293</v>
+      </c>
+      <c r="J24" s="14" t="n">
+        <v>12.72611875397599</v>
+      </c>
       <c r="K24" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -11556,15 +11842,33 @@
           <t>4:8</t>
         </is>
       </c>
-      <c r="B25" s="14" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="14" t="n"/>
-      <c r="I25" s="14" t="n"/>
-      <c r="J25" s="14" t="n"/>
+      <c r="B25" s="14" t="n">
+        <v>0.8416</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>0.722</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>0.6659</v>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>0.6922</v>
+      </c>
+      <c r="F25" s="14" t="n">
+        <v>0.7698</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>0.5017</v>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>0.396</v>
+      </c>
+      <c r="I25" s="14" t="n">
+        <v>0.6556</v>
+      </c>
+      <c r="J25" s="14" t="n">
+        <v>11.53566840666572</v>
+      </c>
       <c r="K25" s="8" t="inlineStr">
         <is>
           <t>N/A</t>
@@ -11645,11 +11949,21 @@
       <c r="J27" s="14" t="n">
         <v>7.855145447281187</v>
       </c>
-      <c r="K27" s="7" t="n"/>
-      <c r="L27" s="7" t="n"/>
-      <c r="M27" s="7" t="n"/>
-      <c r="N27" s="7" t="n"/>
-      <c r="O27" s="7" t="n"/>
+      <c r="K27" s="14" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="L27" s="14" t="n">
+        <v>82.968</v>
+      </c>
+      <c r="M27" s="14" t="n">
+        <v>83.36</v>
+      </c>
+      <c r="N27" s="14" t="n">
+        <v>83.11612778481857</v>
+      </c>
+      <c r="O27" s="14" t="n">
+        <v>84.03603194620464</v>
+      </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
@@ -13181,11 +13495,21 @@
       <c r="J21" s="14" t="n">
         <v>7.855145447281187</v>
       </c>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
-      <c r="O21" s="7" t="n"/>
+      <c r="K21" s="14" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="L21" s="14" t="n">
+        <v>82.968</v>
+      </c>
+      <c r="M21" s="14" t="n">
+        <v>83.36</v>
+      </c>
+      <c r="N21" s="14" t="n">
+        <v>83.11612778481857</v>
+      </c>
+      <c r="O21" s="14" t="n">
+        <v>84.03603194620464</v>
+      </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
@@ -13193,22 +13517,48 @@
           <t>20%</t>
         </is>
       </c>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="14" t="n"/>
-      <c r="E22" s="14" t="n"/>
-      <c r="F22" s="14" t="n"/>
-      <c r="G22" s="14" t="n"/>
-      <c r="H22" s="14" t="n"/>
-      <c r="I22" s="14" t="n"/>
+      <c r="B22" s="14" t="n">
+        <v>0.7813</v>
+      </c>
+      <c r="C22" s="14" t="n">
+        <v>0.8159</v>
+      </c>
+      <c r="D22" s="14" t="n">
+        <v>0.6253</v>
+      </c>
+      <c r="E22" s="14" t="n">
+        <v>0.6882</v>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>0.6987</v>
+      </c>
+      <c r="G22" s="14" t="n">
+        <v>0.4625</v>
+      </c>
+      <c r="H22" s="14" t="n">
+        <v>0.382</v>
+      </c>
+      <c r="I22" s="14" t="n">
+        <v>0.6363</v>
+      </c>
       <c r="J22" s="14" t="n">
         <v>9.555099798748797</v>
       </c>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
-      <c r="N22" s="7" t="n"/>
-      <c r="O22" s="7" t="n"/>
+      <c r="K22" s="14" t="n">
+        <v>73.7</v>
+      </c>
+      <c r="L22" s="14" t="n">
+        <v>72.49399999999999</v>
+      </c>
+      <c r="M22" s="14" t="n">
+        <v>41.36</v>
+      </c>
+      <c r="N22" s="14" t="n">
+        <v>68.76203701117156</v>
+      </c>
+      <c r="O22" s="14" t="n">
+        <v>64.07900925279289</v>
+      </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
@@ -13216,20 +13566,42 @@
           <t>40%</t>
         </is>
       </c>
-      <c r="B23" s="14" t="n"/>
-      <c r="C23" s="14" t="n"/>
-      <c r="D23" s="14" t="n"/>
-      <c r="E23" s="14" t="n"/>
-      <c r="F23" s="14" t="n"/>
-      <c r="G23" s="14" t="n"/>
-      <c r="H23" s="14" t="n"/>
-      <c r="I23" s="14" t="n"/>
+      <c r="B23" s="14" t="n">
+        <v>0.4208</v>
+      </c>
+      <c r="C23" s="14" t="n">
+        <v>0.5306999999999999</v>
+      </c>
+      <c r="D23" s="14" t="n">
+        <v>0.3804</v>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>0.5312</v>
+      </c>
+      <c r="F23" s="14" t="n">
+        <v>0.4024</v>
+      </c>
+      <c r="G23" s="14" t="n">
+        <v>0.2671</v>
+      </c>
+      <c r="H23" s="14" t="n">
+        <v>0.27</v>
+      </c>
+      <c r="I23" s="14" t="n">
+        <v>0.4004</v>
+      </c>
       <c r="J23" s="14" t="n">
         <v>27.57493867845532</v>
       </c>
-      <c r="K23" s="7" t="n"/>
-      <c r="L23" s="7" t="n"/>
-      <c r="M23" s="7" t="n"/>
+      <c r="K23" s="14" t="n">
+        <v>27</v>
+      </c>
+      <c r="L23" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="14" t="n">
+        <v>0</v>
+      </c>
       <c r="N23" s="7" t="n"/>
       <c r="O23" s="7" t="n"/>
     </row>
@@ -13239,20 +13611,42 @@
           <t>50%</t>
         </is>
       </c>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="14" t="n"/>
-      <c r="E24" s="14" t="n"/>
-      <c r="F24" s="14" t="n"/>
-      <c r="G24" s="14" t="n"/>
-      <c r="H24" s="14" t="n"/>
-      <c r="I24" s="14" t="n"/>
+      <c r="B24" s="14" t="n">
+        <v>0.4147</v>
+      </c>
+      <c r="C24" s="14" t="n">
+        <v>0.5018</v>
+      </c>
+      <c r="D24" s="14" t="n">
+        <v>0.2983</v>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>0.5051</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>0.295</v>
+      </c>
+      <c r="G24" s="14" t="n">
+        <v>0.244</v>
+      </c>
+      <c r="H24" s="14" t="n">
+        <v>0.258</v>
+      </c>
+      <c r="I24" s="14" t="n">
+        <v>0.3596</v>
+      </c>
       <c r="J24" s="14" t="n">
         <v>127.0739268153725</v>
       </c>
-      <c r="K24" s="7" t="n"/>
-      <c r="L24" s="7" t="n"/>
-      <c r="M24" s="7" t="n"/>
+      <c r="K24" s="14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="L24" s="14" t="n">
+        <v>0.052</v>
+      </c>
+      <c r="M24" s="14" t="n">
+        <v>0</v>
+      </c>
       <c r="N24" s="7" t="n"/>
       <c r="O24" s="7" t="n"/>
     </row>
@@ -13262,20 +13656,42 @@
           <t>60%</t>
         </is>
       </c>
-      <c r="B25" s="14" t="n"/>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="n"/>
-      <c r="G25" s="14" t="n"/>
-      <c r="H25" s="14" t="n"/>
-      <c r="I25" s="14" t="n"/>
+      <c r="B25" s="14" t="n">
+        <v>0.3783</v>
+      </c>
+      <c r="C25" s="14" t="n">
+        <v>0.5271</v>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>0.2631</v>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>0.5067</v>
+      </c>
+      <c r="F25" s="14" t="n">
+        <v>0.274</v>
+      </c>
+      <c r="G25" s="14" t="n">
+        <v>0.2526</v>
+      </c>
+      <c r="H25" s="14" t="n">
+        <v>0.266</v>
+      </c>
+      <c r="I25" s="14" t="n">
+        <v>0.3525</v>
+      </c>
       <c r="J25" s="14" t="n">
         <v>1341.186220868133</v>
       </c>
-      <c r="K25" s="7" t="n"/>
-      <c r="L25" s="7" t="n"/>
-      <c r="M25" s="7" t="n"/>
+      <c r="K25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="14" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M25" s="14" t="n">
+        <v>0</v>
+      </c>
       <c r="N25" s="7" t="n"/>
       <c r="O25" s="7" t="n"/>
     </row>
@@ -16271,11 +16687,21 @@
       <c r="J21" s="14" t="n">
         <v>7.855145447281187</v>
       </c>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
-      <c r="O21" s="7" t="n"/>
+      <c r="K21" s="14" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="L21" s="14" t="n">
+        <v>82.968</v>
+      </c>
+      <c r="M21" s="14" t="n">
+        <v>83.36</v>
+      </c>
+      <c r="N21" s="14" t="n">
+        <v>83.11612778481857</v>
+      </c>
+      <c r="O21" s="14" t="n">
+        <v>84.03603194620464</v>
+      </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
@@ -16310,11 +16736,21 @@
       <c r="J22" s="14" t="n">
         <v>11.54656722841926</v>
       </c>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
-      <c r="N22" s="7" t="n"/>
-      <c r="O22" s="7" t="n"/>
+      <c r="K22" s="14" t="n">
+        <v>67.7</v>
+      </c>
+      <c r="L22" s="14" t="n">
+        <v>62.956</v>
+      </c>
+      <c r="M22" s="14" t="n">
+        <v>48.64</v>
+      </c>
+      <c r="N22" s="14" t="n">
+        <v>52.20862859347312</v>
+      </c>
+      <c r="O22" s="14" t="n">
+        <v>57.87615714836828</v>
+      </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
@@ -16349,9 +16785,15 @@
       <c r="J23" s="14" t="n">
         <v>43.99941870370173</v>
       </c>
-      <c r="K23" s="7" t="n"/>
-      <c r="L23" s="7" t="n"/>
-      <c r="M23" s="7" t="n"/>
+      <c r="K23" s="14" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="L23" s="14" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="M23" s="14" t="n">
+        <v>0</v>
+      </c>
       <c r="N23" s="7" t="n"/>
       <c r="O23" s="7" t="n"/>
     </row>
@@ -16388,9 +16830,15 @@
       <c r="J24" s="14" t="n">
         <v>200.3270629362775</v>
       </c>
-      <c r="K24" s="7" t="n"/>
-      <c r="L24" s="7" t="n"/>
-      <c r="M24" s="7" t="n"/>
+      <c r="K24" s="14" t="n">
+        <v>10.6</v>
+      </c>
+      <c r="L24" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="14" t="n">
+        <v>0</v>
+      </c>
       <c r="N24" s="7" t="n"/>
       <c r="O24" s="7" t="n"/>
     </row>
@@ -16427,8 +16875,12 @@
       <c r="J25" s="14" t="n">
         <v>1832.389631095462</v>
       </c>
-      <c r="K25" s="7" t="n"/>
-      <c r="L25" s="7" t="n"/>
+      <c r="K25" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="14" t="n">
+        <v>0.005999999999999999</v>
+      </c>
       <c r="M25" s="7" t="n"/>
       <c r="N25" s="7" t="n"/>
       <c r="O25" s="7" t="n"/>
@@ -19425,11 +19877,21 @@
       <c r="J21" s="14" t="n">
         <v>7.855145447281187</v>
       </c>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
-      <c r="O21" s="7" t="n"/>
+      <c r="K21" s="14" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="L21" s="14" t="n">
+        <v>82.968</v>
+      </c>
+      <c r="M21" s="14" t="n">
+        <v>83.36</v>
+      </c>
+      <c r="N21" s="14" t="n">
+        <v>83.11612778481857</v>
+      </c>
+      <c r="O21" s="14" t="n">
+        <v>84.03603194620464</v>
+      </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
@@ -19464,11 +19926,21 @@
       <c r="J22" s="14" t="n">
         <v>11.80012242122977</v>
       </c>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
-      <c r="N22" s="7" t="n"/>
-      <c r="O22" s="7" t="n"/>
+      <c r="K22" s="14" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="L22" s="14" t="n">
+        <v>75.908</v>
+      </c>
+      <c r="M22" s="14" t="n">
+        <v>61.56</v>
+      </c>
+      <c r="N22" s="14" t="n">
+        <v>64.31969449485361</v>
+      </c>
+      <c r="O22" s="14" t="n">
+        <v>69.6219236237134</v>
+      </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
@@ -19503,7 +19975,9 @@
       <c r="J23" s="14" t="n">
         <v>92.03002914120208</v>
       </c>
-      <c r="K23" s="7" t="n"/>
+      <c r="K23" s="14" t="n">
+        <v>12</v>
+      </c>
       <c r="L23" s="7" t="n"/>
       <c r="M23" s="7" t="n"/>
       <c r="N23" s="7" t="n"/>
@@ -22579,11 +23053,21 @@
       <c r="J21" s="14" t="n">
         <v>7.855145447281187</v>
       </c>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
-      <c r="O21" s="7" t="n"/>
+      <c r="K21" s="14" t="n">
+        <v>86.7</v>
+      </c>
+      <c r="L21" s="14" t="n">
+        <v>82.968</v>
+      </c>
+      <c r="M21" s="14" t="n">
+        <v>83.36</v>
+      </c>
+      <c r="N21" s="14" t="n">
+        <v>83.11612778481857</v>
+      </c>
+      <c r="O21" s="14" t="n">
+        <v>84.03603194620464</v>
+      </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="6" t="inlineStr">

</xml_diff>